<commit_message>
Add script to merge clinic dataset files and handle duplicates
- Implemented functionality to load CSV and Excel files from a specified directory.
- Normalized text and phone number formats for consistency.
- Merged datasets while tracking the source file for each entry.
- Identified and separated duplicate entries based on name, address, and phone number.
- Provided options to save deduplicated data and all data including duplicates.
- Output results to CSV and Excel formats.
</commit_message>
<xml_diff>
--- a/clinics/clinic_dataset/dermatologist_in_Kosovo.xlsx
+++ b/clinics/clinic_dataset/dermatologist_in_Kosovo.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J21"/>
+  <dimension ref="A1:J52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -497,7 +497,9 @@
           <t>+383 49 288 433</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr"/>
+      <c r="E2" t="n">
+        <v>104</v>
+      </c>
       <c r="F2" t="n">
         <v>4.9</v>
       </c>
@@ -535,7 +537,9 @@
           <t>+383 45 100 450</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr"/>
+      <c r="E3" t="n">
+        <v>48</v>
+      </c>
       <c r="F3" t="n">
         <v>4.9</v>
       </c>
@@ -573,7 +577,9 @@
           <t>+383 44 161 317</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr"/>
+      <c r="E4" t="n">
+        <v>18</v>
+      </c>
       <c r="F4" t="n">
         <v>3.9</v>
       </c>
@@ -615,7 +621,9 @@
           <t>+383 44 300 298</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr"/>
+      <c r="E5" t="n">
+        <v>87</v>
+      </c>
       <c r="F5" t="n">
         <v>4.3</v>
       </c>
@@ -653,7 +661,9 @@
           <t>+383 44 238 745</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr"/>
+      <c r="E6" t="n">
+        <v>99</v>
+      </c>
       <c r="F6" t="n">
         <v>4.9</v>
       </c>
@@ -695,7 +705,9 @@
           <t>+383 44 159 405</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr"/>
+      <c r="E7" t="n">
+        <v>20</v>
+      </c>
       <c r="F7" t="n">
         <v>5</v>
       </c>
@@ -737,7 +749,9 @@
           <t>+383 46 224 224</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr"/>
+      <c r="E8" t="n">
+        <v>10</v>
+      </c>
       <c r="F8" t="n">
         <v>4.2</v>
       </c>
@@ -779,7 +793,9 @@
           <t>+383 49 263 339</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr"/>
+      <c r="E9" t="n">
+        <v>65</v>
+      </c>
       <c r="F9" t="n">
         <v>4.5</v>
       </c>
@@ -821,7 +837,9 @@
           <t>+383 44 169 327</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr"/>
+      <c r="E10" t="n">
+        <v>5</v>
+      </c>
       <c r="F10" t="n">
         <v>5</v>
       </c>
@@ -845,29 +863,35 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Éclat - Aesthetic Clinic</t>
+          <t>DermaCare</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Jakov Xoxa, Prishtinë 10000</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr"/>
+          <t>14 Ukë Bytyqi, Prishtina 10000</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>http://www.dermacareks.com/</t>
+        </is>
+      </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>+383 49 757 888</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr"/>
+          <t>+383 44 761 000</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>52</v>
+      </c>
       <c r="F11" t="n">
-        <v>4.8</v>
+        <v>4.5</v>
       </c>
       <c r="G11" t="n">
-        <v>42.6470239</v>
+        <v>42.6552983</v>
       </c>
       <c r="H11" t="n">
-        <v>21.1722713</v>
+        <v>21.1658724</v>
       </c>
       <c r="I11" t="inlineStr">
         <is>
@@ -883,33 +907,27 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>DermaCare</t>
+          <t>DuoDerm</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>14 Ukë Bytyqi, Prishtina 10000</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>http://www.dermacareks.com/</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>+383 44 761 000</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr"/>
+          <t>Rr Motrat Qiriazi, Prishtina 10000</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr"/>
+      <c r="D12" t="inlineStr"/>
+      <c r="E12" t="n">
+        <v>5</v>
+      </c>
       <c r="F12" t="n">
-        <v>4.5</v>
+        <v>5</v>
       </c>
       <c r="G12" t="n">
-        <v>42.6552983</v>
+        <v>42.6482963</v>
       </c>
       <c r="H12" t="n">
-        <v>21.1658724</v>
+        <v>21.1601626</v>
       </c>
       <c r="I12" t="inlineStr">
         <is>
@@ -925,25 +943,31 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>DuoDerm</t>
+          <t>Derma R Clinic</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Rr Motrat Qiriazi, Prishtina 10000</t>
+          <t>28 Nëntori, Fushë-Kosovë 10000</t>
         </is>
       </c>
       <c r="C13" t="inlineStr"/>
-      <c r="D13" t="inlineStr"/>
-      <c r="E13" t="inlineStr"/>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>+383 49 157 543</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>2</v>
+      </c>
       <c r="F13" t="n">
         <v>5</v>
       </c>
       <c r="G13" t="n">
-        <v>42.6482963</v>
+        <v>42.6415672</v>
       </c>
       <c r="H13" t="n">
-        <v>21.1601626</v>
+        <v>21.0953951</v>
       </c>
       <c r="I13" t="inlineStr">
         <is>
@@ -959,29 +983,31 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Derma R Clinic</t>
+          <t>Asa Medical Aesthetics</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>28 Nëntori, Fushë-Kosovë 10000</t>
+          <t>Rruga B, Prishtinë 10000</t>
         </is>
       </c>
       <c r="C14" t="inlineStr"/>
       <c r="D14" t="inlineStr">
         <is>
-          <t>+383 49 157 543</t>
-        </is>
-      </c>
-      <c r="E14" t="inlineStr"/>
+          <t>+383 49 293 747</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>65</v>
+      </c>
       <c r="F14" t="n">
-        <v>5</v>
+        <v>4.6</v>
       </c>
       <c r="G14" t="n">
-        <v>42.6415672</v>
+        <v>42.6522425</v>
       </c>
       <c r="H14" t="n">
-        <v>21.0953951</v>
+        <v>21.1771033</v>
       </c>
       <c r="I14" t="inlineStr">
         <is>
@@ -997,31 +1023,31 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Kirurgjia estetike italiane Prishtine - DaVINCI</t>
+          <t>Éclat - Aesthetic Clinic</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Jusuf Gervalla, Lagja, Prishtinë 10000</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>http://www.davinci.al/</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr"/>
+          <t>Jakov Xoxa, Prishtinë 10000</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr"/>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>+383 49 757 888</t>
+        </is>
+      </c>
       <c r="E15" t="n">
-        <v>173</v>
+        <v>19</v>
       </c>
       <c r="F15" t="n">
-        <v>4.9</v>
+        <v>4.8</v>
       </c>
       <c r="G15" t="n">
-        <v>42.6494541</v>
+        <v>42.6470239</v>
       </c>
       <c r="H15" t="n">
-        <v>21.1507998</v>
+        <v>21.1722713</v>
       </c>
       <c r="I15" t="inlineStr">
         <is>
@@ -1037,29 +1063,35 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Asa Medical Aesthetics</t>
+          <t>Anaderm Aesthetic Surgery Hospital</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Rruga B, Prishtinë 10000</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr"/>
+          <t>Prishtinë , Kosovo, Street Zef Jubani, Prishtina 10000</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>https://www.klinikaanaderm.com/</t>
+        </is>
+      </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>+383 49 293 747</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr"/>
+          <t>+383 45 707 744</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
+        <v>73</v>
+      </c>
       <c r="F16" t="n">
-        <v>4.6</v>
+        <v>4.8</v>
       </c>
       <c r="G16" t="n">
-        <v>42.6522425</v>
+        <v>42.631382</v>
       </c>
       <c r="H16" t="n">
-        <v>21.1771033</v>
+        <v>21.1484613</v>
       </c>
       <c r="I16" t="inlineStr">
         <is>
@@ -1075,33 +1107,31 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Anaderm Aesthetic Surgery Hospital</t>
+          <t>Kirurgjia estetike italiane Prishtine - DaVINCI</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Prishtinë , Kosovo, Street Zef Jubani, Prishtina 10000</t>
+          <t>Jusuf Gervalla, Lagja, Prishtinë 10000</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>https://www.klinikaanaderm.com/</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>+383 45 707 744</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr"/>
+          <t>http://www.davinci.al/</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr"/>
+      <c r="E17" t="n">
+        <v>173</v>
+      </c>
       <c r="F17" t="n">
-        <v>4.8</v>
+        <v>4.9</v>
       </c>
       <c r="G17" t="n">
-        <v>42.631382</v>
+        <v>42.6494541</v>
       </c>
       <c r="H17" t="n">
-        <v>21.1484613</v>
+        <v>21.1507998</v>
       </c>
       <c r="I17" t="inlineStr">
         <is>
@@ -1117,33 +1147,31 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Miliona Aesthetic</t>
+          <t>Ordinanca Dermatologjike DermaMegi</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Rruga B, Prishtinë 10000</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>http://miliona.com/</t>
-        </is>
-      </c>
+          <t>M54M+863, Prishtinë 10000</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr"/>
       <c r="D18" t="inlineStr">
         <is>
-          <t>+383 44 911 222</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr"/>
+          <t>+377 44 238 750</t>
+        </is>
+      </c>
+      <c r="E18" t="n">
+        <v>7</v>
+      </c>
       <c r="F18" t="n">
-        <v>4.6</v>
+        <v>3.1</v>
       </c>
       <c r="G18" t="n">
-        <v>42.6550665</v>
+        <v>42.6557643</v>
       </c>
       <c r="H18" t="n">
-        <v>21.1782976</v>
+        <v>21.1830553</v>
       </c>
       <c r="I18" t="inlineStr">
         <is>
@@ -1159,29 +1187,35 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Ordinanca Dermatologjike DermaMegi</t>
+          <t>Miliona Aesthetic</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>M54M+863, Prishtinë 10000</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr"/>
+          <t>Rruga B, Prishtinë 10000</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>http://miliona.com/</t>
+        </is>
+      </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>+377 44 238 750</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr"/>
+          <t>+383 44 911 222</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>84</v>
+      </c>
       <c r="F19" t="n">
-        <v>3.1</v>
+        <v>4.6</v>
       </c>
       <c r="G19" t="n">
-        <v>42.6557643</v>
+        <v>42.6550665</v>
       </c>
       <c r="H19" t="n">
-        <v>21.1830553</v>
+        <v>21.1782976</v>
       </c>
       <c r="I19" t="inlineStr">
         <is>
@@ -1197,25 +1231,35 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Klinika e Dermatovenerologjisë</t>
+          <t>estethica</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>10000 Unnamed Road, Prishtinë 10000</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr"/>
-      <c r="D20" t="inlineStr"/>
-      <c r="E20" t="inlineStr"/>
+          <t>30 Rrugë Nekibe Kelmendi, Prishtinë 10000</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>http://www.estethica-ks.com/</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>+383 49 660 660</t>
+        </is>
+      </c>
+      <c r="E20" t="n">
+        <v>1206</v>
+      </c>
       <c r="F20" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="G20" t="n">
-        <v>42.6433131</v>
+        <v>42.6299485</v>
       </c>
       <c r="H20" t="n">
-        <v>21.1646911</v>
+        <v>21.1608969</v>
       </c>
       <c r="I20" t="inlineStr">
         <is>
@@ -1231,42 +1275,1290 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
+          <t>Klinika e Dermatovenerologjisë</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>10000 Unnamed Road, Prishtinë 10000</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr"/>
+      <c r="D21" t="inlineStr"/>
+      <c r="E21" t="n">
+        <v>1</v>
+      </c>
+      <c r="F21" t="n">
+        <v>1</v>
+      </c>
+      <c r="G21" t="n">
+        <v>42.6433131</v>
+      </c>
+      <c r="H21" t="n">
+        <v>21.1646911</v>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>dermatologist</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>Kosovo</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Poliklinika SHOSHI</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Kodra e Diellit, Rr. Rifat Burgjeviq Hyrja 8 Nr. 1. (afër Qendrës Tregtare) Prishtinë, Hyrja 8 Nr. 1. Rifat Burdzeviç, Prishtinë 10000</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr"/>
+      <c r="D22" t="inlineStr"/>
+      <c r="E22" t="n">
+        <v>18</v>
+      </c>
+      <c r="F22" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="G22" t="n">
+        <v>42.6520832</v>
+      </c>
+      <c r="H22" t="n">
+        <v>21.1671185</v>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>dermatologist</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>Kosovo</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>TrueLife Clinic</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Rruga B, Prishtinë 10000</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr"/>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>+383 48 811 555</t>
+        </is>
+      </c>
+      <c r="E23" t="n">
+        <v>21</v>
+      </c>
+      <c r="F23" t="n">
+        <v>5</v>
+      </c>
+      <c r="G23" t="n">
+        <v>42.6496501</v>
+      </c>
+      <c r="H23" t="n">
+        <v>21.1738625</v>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>dermatologist</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>Kosovo</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
           <t>American Beauty Clinic</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
+      <c r="B24" t="inlineStr">
         <is>
           <t>Agi Kos, Nr c2, Objekti 3, Rruga Vicianum, lokali4.1 2, Prishtinë 10000</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
+      <c r="C24" t="inlineStr">
         <is>
           <t>https://americanbeautyclinic.com/</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr">
+      <c r="D24" t="inlineStr">
         <is>
           <t>+383 48 596 596</t>
         </is>
       </c>
-      <c r="E21" t="n">
+      <c r="E24" t="n">
         <v>10</v>
       </c>
-      <c r="F21" t="n">
+      <c r="F24" t="n">
         <v>5</v>
       </c>
-      <c r="G21" t="n">
+      <c r="G24" t="n">
         <v>42.6605313</v>
       </c>
-      <c r="H21" t="n">
+      <c r="H24" t="n">
         <v>21.1509951</v>
       </c>
-      <c r="I21" t="inlineStr">
-        <is>
-          <t>dermatologist</t>
-        </is>
-      </c>
-      <c r="J21" t="inlineStr">
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>dermatologist</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>Kosovo</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>ECHO MED Qendra Diagnostike Terapeutike</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>nr. 3 Rruga Xheladin Kurbaliu, Prishtinë 10000</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr"/>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>+383 44 734 394</t>
+        </is>
+      </c>
+      <c r="E25" t="n">
+        <v>1</v>
+      </c>
+      <c r="F25" t="inlineStr"/>
+      <c r="G25" t="n">
+        <v>42.6680951</v>
+      </c>
+      <c r="H25" t="n">
+        <v>21.1701668</v>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>dermatologist</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>Kosovo</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>University Clinical Center of Kosovo</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>J5V6+98V, Prishtinë 10000</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>https://shskuk.rks-gov.net/QKUK/QKUK/historikuQKUK</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>+381 38 500600</t>
+        </is>
+      </c>
+      <c r="E26" t="n">
+        <v>89</v>
+      </c>
+      <c r="F26" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="G26" t="n">
+        <v>42.6434827</v>
+      </c>
+      <c r="H26" t="n">
+        <v>21.1607975</v>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>dermatologist</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>Kosovo</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>To Fill Clinic</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Rruga Ferid Curri, Prishtinë 10000</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/profile.php?id=100087602140996</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>+383 45 717 873</t>
+        </is>
+      </c>
+      <c r="E27" t="n">
+        <v>10</v>
+      </c>
+      <c r="F27" t="n">
+        <v>5</v>
+      </c>
+      <c r="G27" t="n">
+        <v>42.6598176</v>
+      </c>
+      <c r="H27" t="n">
+        <v>21.139417</v>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>dermatologist</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>Kosovo</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Rare Clinic Aesthetic</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Nënë Tereza, Fushë-Kosovë 12000</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr"/>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>+383 48 511 955</t>
+        </is>
+      </c>
+      <c r="E28" t="n">
+        <v>18</v>
+      </c>
+      <c r="F28" t="n">
+        <v>5</v>
+      </c>
+      <c r="G28" t="n">
+        <v>42.6422579</v>
+      </c>
+      <c r="H28" t="n">
+        <v>21.1099006</v>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>dermatologist</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>Kosovo</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Este Medical Kosova</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Shkup, km, Magjistralja, 3, Prishtinë 10000</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>https://www.estemedicalgroup.al/</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>+383 48 384 384</t>
+        </is>
+      </c>
+      <c r="E29" t="n">
+        <v>10</v>
+      </c>
+      <c r="F29" t="n">
+        <v>5</v>
+      </c>
+      <c r="G29" t="n">
+        <v>42.6060201</v>
+      </c>
+      <c r="H29" t="n">
+        <v>21.1359354</v>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>dermatologist</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>Kosovo</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>EEV Group</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Agim Ramadani, Prishtinë 10000</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>https://eevgroupks.com/</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr"/>
+      <c r="E30" t="n">
+        <v>2</v>
+      </c>
+      <c r="F30" t="n">
+        <v>5</v>
+      </c>
+      <c r="G30" t="n">
+        <v>42.6610501</v>
+      </c>
+      <c r="H30" t="n">
+        <v>21.1648029</v>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>dermatologist</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>Kosovo</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Emergency</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>3 Stomatologjia, Prishtinë 10000</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr"/>
+      <c r="D31" t="inlineStr"/>
+      <c r="E31" t="n">
+        <v>4</v>
+      </c>
+      <c r="F31" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="G31" t="n">
+        <v>42.6451936</v>
+      </c>
+      <c r="H31" t="n">
+        <v>21.1622295</v>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>dermatologist</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>Kosovo</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>American Clinic - Dr.Behar Kusari</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>M2, Çagllavicë, Prishtinë 10000</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>http://american-art.net/</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>+383 44 126 188</t>
+        </is>
+      </c>
+      <c r="E32" t="n">
+        <v>125</v>
+      </c>
+      <c r="F32" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="G32" t="n">
+        <v>42.6204039</v>
+      </c>
+      <c r="H32" t="n">
+        <v>21.1445569</v>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>dermatologist</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>Kosovo</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Hana Dermatology Estetic</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr"/>
+      <c r="C33" t="inlineStr"/>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>+383 44 440 050</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr"/>
+      <c r="F33" t="inlineStr"/>
+      <c r="G33" t="n">
+        <v>42.6663801</v>
+      </c>
+      <c r="H33" t="n">
+        <v>21.1587273</v>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>dermatologist</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>Kosovo</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Anaderm</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Rr, 33, 1 Hilmi Rakovica, Prishtinë</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr"/>
+      <c r="D34" t="inlineStr"/>
+      <c r="E34" t="n">
+        <v>1</v>
+      </c>
+      <c r="F34" t="n">
+        <v>1</v>
+      </c>
+      <c r="G34" t="n">
+        <v>42.652786</v>
+      </c>
+      <c r="H34" t="n">
+        <v>21.1706923</v>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>dermatologist</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>Kosovo</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Dr. Vivien</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Bill Clinton, Prishtinë 10000</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr"/>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>+383 44 762 312</t>
+        </is>
+      </c>
+      <c r="E35" t="n">
+        <v>2</v>
+      </c>
+      <c r="F35" t="n">
+        <v>5</v>
+      </c>
+      <c r="G35" t="n">
+        <v>42.65479</v>
+      </c>
+      <c r="H35" t="n">
+        <v>21.153817</v>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>dermatologist</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>Kosovo</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>DOKTORI JUAJ</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Ali Vitia, Prishtinë 10000</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>https://doktorijuaj.com/</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>+383 44 444 752</t>
+        </is>
+      </c>
+      <c r="E36" t="n">
+        <v>5</v>
+      </c>
+      <c r="F36" t="n">
+        <v>5</v>
+      </c>
+      <c r="G36" t="n">
+        <v>42.6376698</v>
+      </c>
+      <c r="H36" t="n">
+        <v>21.1531732</v>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>dermatologist</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>Kosovo</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Derma Aesthetic Center by Ndricimi-RM</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Rruga Çameria Nr:6 Rru, Pejë 30000</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr"/>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>+383 48 222 977</t>
+        </is>
+      </c>
+      <c r="E37" t="n">
+        <v>4</v>
+      </c>
+      <c r="F37" t="n">
+        <v>5</v>
+      </c>
+      <c r="G37" t="n">
+        <v>42.6621038</v>
+      </c>
+      <c r="H37" t="n">
+        <v>20.2877494</v>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>dermatologist</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>Kosovo</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>TITI HAIR CLINIC</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Sllatine e madhe, Fushe</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr"/>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>+383 49 337 300</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr"/>
+      <c r="F38" t="inlineStr"/>
+      <c r="G38" t="n">
+        <v>42.5986532</v>
+      </c>
+      <c r="H38" t="n">
+        <v>21.0210462</v>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>dermatologist</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>Kosovo</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Dardanica Clinic SH.P.K.</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Muhamet Çami, Prishtinë 10000</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>http://www.dardanica-clinic.com/</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>+383 45 448 822</t>
+        </is>
+      </c>
+      <c r="E39" t="n">
+        <v>6</v>
+      </c>
+      <c r="F39" t="n">
+        <v>5</v>
+      </c>
+      <c r="G39" t="n">
+        <v>42.6433536</v>
+      </c>
+      <c r="H39" t="n">
+        <v>21.169272</v>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>dermatologist</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>Kosovo</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Derma Clinic Dr. Dafina Ibrahimi-Devaja</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>FF5C+JRM, Gjilan 60000</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/DermaClinicDA/</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>+383 45 969 270</t>
+        </is>
+      </c>
+      <c r="E40" t="n">
+        <v>1</v>
+      </c>
+      <c r="F40" t="n">
+        <v>5</v>
+      </c>
+      <c r="G40" t="n">
+        <v>42.4590828</v>
+      </c>
+      <c r="H40" t="n">
+        <v>21.4720451</v>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>dermatologist</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>Kosovo</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Derma Pure</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Wesley Clark, Pejë 30000</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/dermapure.clinicks</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>+383 49 164 343</t>
+        </is>
+      </c>
+      <c r="E41" t="n">
+        <v>30</v>
+      </c>
+      <c r="F41" t="n">
+        <v>4.9</v>
+      </c>
+      <c r="G41" t="n">
+        <v>42.6610654</v>
+      </c>
+      <c r="H41" t="n">
+        <v>20.2808265</v>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>dermatologist</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>Kosovo</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Estetika skin</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>rruga ali hajdari, Gjilan</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr"/>
+      <c r="D42" t="inlineStr"/>
+      <c r="E42" t="n">
+        <v>1</v>
+      </c>
+      <c r="F42" t="n">
+        <v>5</v>
+      </c>
+      <c r="G42" t="n">
+        <v>42.4690305</v>
+      </c>
+      <c r="H42" t="n">
+        <v>21.4622439</v>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>dermatologist</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>Kosovo</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Vioderm</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Rruga Emin Duraku, Ferizaj 70000</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr"/>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>+383 45 120 020</t>
+        </is>
+      </c>
+      <c r="E43" t="n">
+        <v>2</v>
+      </c>
+      <c r="F43" t="n">
+        <v>5</v>
+      </c>
+      <c r="G43" t="n">
+        <v>42.3732033</v>
+      </c>
+      <c r="H43" t="n">
+        <v>21.1565401</v>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>dermatologist</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>Kosovo</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Poliklinika Uro-Med</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Fatmir Ratkoceri, Ferizaj 70000</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr"/>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>+383 45 324 000</t>
+        </is>
+      </c>
+      <c r="E44" t="n">
+        <v>11</v>
+      </c>
+      <c r="F44" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="G44" t="n">
+        <v>42.3811136</v>
+      </c>
+      <c r="H44" t="n">
+        <v>21.15353</v>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>dermatologist</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>Kosovo</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Dermatovenerolog Mujadin Tërshnjaku(Estetika)</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Rr William Walker, Prizren 20000</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr"/>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>+383 44 315 413</t>
+        </is>
+      </c>
+      <c r="E45" t="n">
+        <v>2</v>
+      </c>
+      <c r="F45" t="n">
+        <v>5</v>
+      </c>
+      <c r="G45" t="n">
+        <v>42.2079321</v>
+      </c>
+      <c r="H45" t="n">
+        <v>20.7246258</v>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>dermatologist</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>Kosovo</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>EPIDERMIS - Advanced Aesthetics</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Driton Islami, Ferizaj 70000</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr"/>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>+383 49 100 183</t>
+        </is>
+      </c>
+      <c r="E46" t="n">
+        <v>3</v>
+      </c>
+      <c r="F46" t="n">
+        <v>5</v>
+      </c>
+      <c r="G46" t="n">
+        <v>42.3771097</v>
+      </c>
+      <c r="H46" t="n">
+        <v>21.1408827</v>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>dermatologist</t>
+        </is>
+      </c>
+      <c r="J46" t="inlineStr">
+        <is>
+          <t>Kosovo</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>Poliklinika Fati- Vushtrri</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Gjon Buzuku, Vushtrri 42000</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr"/>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>+383 49 818 144</t>
+        </is>
+      </c>
+      <c r="E47" t="n">
+        <v>2</v>
+      </c>
+      <c r="F47" t="n">
+        <v>5</v>
+      </c>
+      <c r="G47" t="n">
+        <v>42.8218465</v>
+      </c>
+      <c r="H47" t="n">
+        <v>20.974281</v>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>dermatologist</t>
+        </is>
+      </c>
+      <c r="J47" t="inlineStr">
+        <is>
+          <t>Kosovo</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Ordinanca Dermatologjike “Derma”</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>p.n Gjon Buzuku, Skënderaj 41000</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/p/Ordinanca-Dermatologjike-Derma-100063816504152/</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>+383 44 196 143</t>
+        </is>
+      </c>
+      <c r="E48" t="n">
+        <v>3</v>
+      </c>
+      <c r="F48" t="inlineStr"/>
+      <c r="G48" t="n">
+        <v>42.7493588</v>
+      </c>
+      <c r="H48" t="n">
+        <v>20.7902115</v>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>dermatologist</t>
+        </is>
+      </c>
+      <c r="J48" t="inlineStr">
+        <is>
+          <t>Kosovo</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>Poliklinika Beni</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Bedri Pejani, Vushtrri 42000</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr"/>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>+383 44 732 162</t>
+        </is>
+      </c>
+      <c r="E49" t="n">
+        <v>1</v>
+      </c>
+      <c r="F49" t="n">
+        <v>5</v>
+      </c>
+      <c r="G49" t="n">
+        <v>42.8236334</v>
+      </c>
+      <c r="H49" t="n">
+        <v>20.9631371</v>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>dermatologist</t>
+        </is>
+      </c>
+      <c r="J49" t="inlineStr">
+        <is>
+          <t>Kosovo</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>Fiziomed</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Nysret Seharsoj, Prizren 20000</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>http://www.fiziomed.com/</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>+383 44 366 009</t>
+        </is>
+      </c>
+      <c r="E50" t="n">
+        <v>16</v>
+      </c>
+      <c r="F50" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="G50" t="n">
+        <v>42.2058716</v>
+      </c>
+      <c r="H50" t="n">
+        <v>20.7318058</v>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>dermatologist</t>
+        </is>
+      </c>
+      <c r="J50" t="inlineStr">
+        <is>
+          <t>Kosovo</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>Ordinanca për sëmundje të lëkurës Dr Arsim Riza “Leta”</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>114 Deshmoret e Lirise, Gjakova 50000</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr"/>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>+383 44 247 327</t>
+        </is>
+      </c>
+      <c r="E51" t="n">
+        <v>1</v>
+      </c>
+      <c r="F51" t="n">
+        <v>5</v>
+      </c>
+      <c r="G51" t="n">
+        <v>42.3705377</v>
+      </c>
+      <c r="H51" t="n">
+        <v>20.4305078</v>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>dermatologist</t>
+        </is>
+      </c>
+      <c r="J51" t="inlineStr">
+        <is>
+          <t>Kosovo</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>iDerm</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>65 Azem Bejta, Prizren 20000</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/idermpz</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>+383 44 515 105</t>
+        </is>
+      </c>
+      <c r="E52" t="n">
+        <v>9</v>
+      </c>
+      <c r="F52" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="G52" t="n">
+        <v>42.2135357</v>
+      </c>
+      <c r="H52" t="n">
+        <v>20.7322064</v>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>dermatologist</t>
+        </is>
+      </c>
+      <c r="J52" t="inlineStr">
         <is>
           <t>Kosovo</t>
         </is>

</xml_diff>